<commit_message>
Feat: Expand to 20 tests (fix TC-04/11/14, add TC-16..20 for input validation, multi-dept, and session logic)
</commit_message>
<xml_diff>
--- a/tests/TC-01/results/unscheduled_courses_even.xlsx
+++ b/tests/TC-01/results/unscheduled_courses_even.xlsx
@@ -862,12 +862,12 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>LAB</t>
+          <t>LEC, LAB</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>No computer lab available (Needs 50 capacity)</t>
+          <t>Could not find suitable slot (Needs 50 capacity); No computer lab available (Needs 50 capacity)</t>
         </is>
       </c>
     </row>

</xml_diff>